<commit_message>
Add willingness-to-pay filter for the proposed $100k setup / $30k/mo ticket
New section in Resumen: computes minimum annual revenue needed for the
ticket to stay under a comfortable % of revenue, references the legal
MIPYME revenue bands added to Fuentes, and applies an explicitly-flagged
assumption (35%, the weakest-grounded number in the model) to size how
much of the existing SOM can plausibly afford it.
</commit_message>
<xml_diff>
--- a/modelo-mercado-pymes-mexico.xlsx
+++ b/modelo-mercado-pymes-mexico.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="117">
   <si>
     <t xml:space="preserve">Fuentes y supuestos — modelo de mercado de PYMEs en México</t>
   </si>
@@ -173,6 +173,21 @@
     <t xml:space="preserve">Leyenda: texto azul = dato/insumo fijo tomado de la fuente citada. Relleno amarillo + texto azul = SUPUESTO editable (cámbialo aquí; el resto del modelo usa esta misma celda). Texto negro = resultado calculado con fórmula.</t>
   </si>
   <si>
+    <t xml:space="preserve">Datos adicionales — banda legal de ingresos anuales por tamaño de empresa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Piso de ingresos anuales — Pequeña empresa (millones de pesos)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Estratificación oficial MIPYME (Ley para el Desarrollo de la Competitividad de la MIPYME / Acuerdo DOF)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Techo de Pequeña empresa / piso de Mediana empresa (millones de pesos)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Techo de Mediana empresa (millones de pesos)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Vía A — Servicios que cotizan proyecto por proyecto (diseño, consultoría, arquitectura, construcción)</t>
   </si>
   <si>
@@ -294,6 +309,42 @@
   </si>
   <si>
     <t xml:space="preserve">Prospectar primero en Ciudad de México y Estado de México reduce fricción logística: concentran cerca de una quinta parte de los servicios profesionales del país. No hay un dato equivalente citado aquí para la concentración geográfica de restaurantes (Vía B).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">¿Cuántos pueden pagar el ticket propuesto ($100,000 setup + $30,000/mes)?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Setup propuesto (MXN)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mensualidad propuesta (MXN)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Costo total año 1 (setup + 12 meses de mensualidad)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Costo anual recurrente (año 2 en adelante)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">% de ingresos anuales que representa un gasto "cómodo" — no una carga desproporcionada (umbral, supuesto)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ingreso anual mínimo para que el costo del año 1 sea ≤ umbral</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ingreso anual mínimo para sostener el costo recurrente ≤ umbral</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Referencia — banda legal de ingresos anuales: Pequeña empresa $4.01–100 millones de pesos/año; Mediana empresa $100.01–250 millones de pesos/año (ver hoja 'Fuentes'). El ingreso mínimo recurrente calculado arriba cae dentro del tramo bajo de 'Pequeña' — es decir, una parte real pero no total de las empresas ya filtradas como Pequeña/Mediana puede sostenerlo sin que sea una carga desproporcionada.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">% del mercado obtenible (SOM) que se estima tiene ingresos suficientes para pagar este ticket cómodamente (supuesto)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MERCADO QUE PUEDE PAGAR EL TICKET PROPUESTO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nota: el 35% es la cifra menos sólida de todo el modelo — no encontré una distribución pública de ingresos DENTRO de la banda Pequeña/Mediana en México (esa banda va de $4M a $250M/año, un rango enorme). Es una estimación de sentido común, no un dato censal. El punto de referencia más confiable que existe es tu cliente actual: compara qué % de sus ingresos representa lo que le cobras hoy, y ajusta esta celda con ese punto de anclaje real.</t>
   </si>
   <si>
     <t xml:space="preserve">Sensibilidad — 3 escenarios</t>
@@ -330,13 +381,14 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="#,##0"/>
     <numFmt numFmtId="166" formatCode="0.0%"/>
     <numFmt numFmtId="167" formatCode="#,##0.0"/>
+    <numFmt numFmtId="168" formatCode="\$#,##0"/>
   </numFmts>
-  <fonts count="17">
+  <fonts count="19">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -432,6 +484,14 @@
     <font>
       <b val="true"/>
       <sz val="11"/>
+      <color rgb="FF1F1F1F"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="0"/>
@@ -457,6 +517,14 @@
       <b val="true"/>
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <i val="true"/>
+      <sz val="9"/>
+      <color rgb="FF7A5B00"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -537,7 +605,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="38">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -594,19 +662,27 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -614,11 +690,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="13" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="14" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="14" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -626,15 +702,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="16" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="17" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="17" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -642,7 +718,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -658,8 +734,24 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="13" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="167" fontId="14" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
@@ -918,7 +1010,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D31"/>
+  <dimension ref="A1:D36"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="58"/>
@@ -1296,12 +1388,63 @@
       <c r="C31" s="13"/>
       <c r="D31" s="13"/>
     </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="14" t="s">
+        <v>49</v>
+      </c>
+      <c r="B33" s="14"/>
+      <c r="C33" s="14"/>
+      <c r="D33" s="14"/>
+    </row>
+    <row r="34" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="B34" s="15" t="n">
+        <v>4.01</v>
+      </c>
+      <c r="C34" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="D34" s="7" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="B35" s="15" t="n">
+        <v>100</v>
+      </c>
+      <c r="C35" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="D35" s="7" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="B36" s="15" t="n">
+        <v>250</v>
+      </c>
+      <c r="C36" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="D36" s="7" t="s">
+        <v>51</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="5">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A2:D2"/>
     <mergeCell ref="A26:D26"/>
     <mergeCell ref="A31:D31"/>
+    <mergeCell ref="A33:D33"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -1329,7 +1472,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1337,7 +1480,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -1345,110 +1488,110 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>3</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="14" t="n">
+      <c r="A5" s="16" t="n">
         <v>1</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="C5" s="15" t="n">
+        <v>59</v>
+      </c>
+      <c r="C5" s="17" t="n">
         <f aca="false">Fuentes!$B$17</f>
         <v>109630</v>
       </c>
-      <c r="D5" s="16" t="s">
-        <v>55</v>
+      <c r="D5" s="18" t="s">
+        <v>60</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="14" t="n">
+      <c r="A6" s="16" t="n">
         <v>2</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="C6" s="17" t="n">
+        <v>61</v>
+      </c>
+      <c r="C6" s="19" t="n">
         <f aca="false">Fuentes!$B$27</f>
         <v>0.25</v>
       </c>
-      <c r="D6" s="16" t="s">
-        <v>57</v>
+      <c r="D6" s="18" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="18"/>
-      <c r="B7" s="19" t="s">
-        <v>58</v>
-      </c>
-      <c r="C7" s="20" t="n">
+      <c r="A7" s="20"/>
+      <c r="B7" s="21" t="s">
+        <v>63</v>
+      </c>
+      <c r="C7" s="22" t="n">
         <f aca="false">C5*C6</f>
         <v>27407.5</v>
       </c>
-      <c r="D7" s="18"/>
+      <c r="D7" s="20"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="14" t="n">
+      <c r="A8" s="16" t="n">
         <v>3</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="C8" s="17" t="n">
+        <v>64</v>
+      </c>
+      <c r="C8" s="19" t="n">
         <f aca="false">Fuentes!$B$28</f>
         <v>0.85</v>
       </c>
-      <c r="D8" s="16" t="s">
-        <v>60</v>
+      <c r="D8" s="18" t="s">
+        <v>65</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="18"/>
-      <c r="B9" s="19" t="s">
-        <v>61</v>
-      </c>
-      <c r="C9" s="20" t="n">
+      <c r="A9" s="20"/>
+      <c r="B9" s="21" t="s">
+        <v>66</v>
+      </c>
+      <c r="C9" s="22" t="n">
         <f aca="false">C7*C8</f>
         <v>23296.375</v>
       </c>
-      <c r="D9" s="18"/>
+      <c r="D9" s="20"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="14" t="n">
+      <c r="A10" s="16" t="n">
         <v>4</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>62</v>
-      </c>
-      <c r="C10" s="17" t="n">
+        <v>67</v>
+      </c>
+      <c r="C10" s="19" t="n">
         <f aca="false">Fuentes!$B$29</f>
         <v>0.2</v>
       </c>
-      <c r="D10" s="16" t="s">
-        <v>60</v>
+      <c r="D10" s="18" t="s">
+        <v>65</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="21"/>
-      <c r="B11" s="22" t="s">
-        <v>63</v>
-      </c>
-      <c r="C11" s="23" t="n">
+      <c r="A11" s="23"/>
+      <c r="B11" s="24" t="s">
+        <v>68</v>
+      </c>
+      <c r="C11" s="25" t="n">
         <f aca="false">C9*C10</f>
         <v>4659.275</v>
       </c>
-      <c r="D11" s="21"/>
+      <c r="D11" s="23"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -1481,7 +1624,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1489,7 +1632,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -1497,110 +1640,110 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>3</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="14" t="n">
+      <c r="A5" s="16" t="n">
         <v>1</v>
       </c>
       <c r="B5" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="C5" s="15" t="n">
+      <c r="C5" s="17" t="n">
         <f aca="false">Fuentes!$B$14</f>
         <v>641000</v>
       </c>
-      <c r="D5" s="16" t="s">
-        <v>55</v>
+      <c r="D5" s="18" t="s">
+        <v>60</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="14" t="n">
+      <c r="A6" s="16" t="n">
         <v>2</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>65</v>
-      </c>
-      <c r="C6" s="17" t="n">
+        <v>70</v>
+      </c>
+      <c r="C6" s="19" t="n">
         <f aca="false">Fuentes!$B$16</f>
         <v>0.04</v>
       </c>
-      <c r="D6" s="16" t="s">
-        <v>57</v>
+      <c r="D6" s="18" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="18"/>
-      <c r="B7" s="19" t="s">
-        <v>58</v>
-      </c>
-      <c r="C7" s="20" t="n">
+      <c r="A7" s="20"/>
+      <c r="B7" s="21" t="s">
+        <v>63</v>
+      </c>
+      <c r="C7" s="22" t="n">
         <f aca="false">C5*C6</f>
         <v>25640</v>
       </c>
-      <c r="D7" s="18"/>
+      <c r="D7" s="20"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="14" t="n">
+      <c r="A8" s="16" t="n">
         <v>3</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="C8" s="17" t="n">
+        <v>64</v>
+      </c>
+      <c r="C8" s="19" t="n">
         <f aca="false">Fuentes!$B$28</f>
         <v>0.85</v>
       </c>
-      <c r="D8" s="16" t="s">
-        <v>60</v>
+      <c r="D8" s="18" t="s">
+        <v>65</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="18"/>
-      <c r="B9" s="19" t="s">
-        <v>61</v>
-      </c>
-      <c r="C9" s="20" t="n">
+      <c r="A9" s="20"/>
+      <c r="B9" s="21" t="s">
+        <v>66</v>
+      </c>
+      <c r="C9" s="22" t="n">
         <f aca="false">C7*C8</f>
         <v>21794</v>
       </c>
-      <c r="D9" s="18"/>
+      <c r="D9" s="20"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="14" t="n">
+      <c r="A10" s="16" t="n">
         <v>4</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>62</v>
-      </c>
-      <c r="C10" s="17" t="n">
+        <v>67</v>
+      </c>
+      <c r="C10" s="19" t="n">
         <f aca="false">Fuentes!$B$29</f>
         <v>0.2</v>
       </c>
-      <c r="D10" s="16" t="s">
-        <v>60</v>
+      <c r="D10" s="18" t="s">
+        <v>65</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="21"/>
-      <c r="B11" s="22" t="s">
-        <v>66</v>
-      </c>
-      <c r="C11" s="23" t="n">
+      <c r="A11" s="23"/>
+      <c r="B11" s="24" t="s">
+        <v>71</v>
+      </c>
+      <c r="C11" s="25" t="n">
         <f aca="false">C9*C10</f>
         <v>4358.8</v>
       </c>
-      <c r="D11" s="21"/>
+      <c r="D11" s="23"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -1622,7 +1765,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E28"/>
+  <dimension ref="A1:E43"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="46"/>
@@ -1632,7 +1775,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1641,7 +1784,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -1649,50 +1792,50 @@
       <c r="E2" s="2"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="24" t="s">
-        <v>69</v>
-      </c>
-      <c r="B4" s="24"/>
+      <c r="A4" s="26" t="s">
+        <v>74</v>
+      </c>
+      <c r="B4" s="26"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="25" t="s">
-        <v>70</v>
-      </c>
-      <c r="B5" s="26" t="n">
+      <c r="A5" s="27" t="s">
+        <v>75</v>
+      </c>
+      <c r="B5" s="28" t="n">
         <f aca="false">'Via A'!C11</f>
         <v>4659.275</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="25" t="s">
-        <v>71</v>
-      </c>
-      <c r="B6" s="26" t="n">
+      <c r="A6" s="27" t="s">
+        <v>76</v>
+      </c>
+      <c r="B6" s="28" t="n">
         <f aca="false">'Via B'!C11</f>
         <v>4358.8</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="22" t="s">
-        <v>72</v>
-      </c>
-      <c r="B7" s="23" t="n">
+      <c r="A7" s="24" t="s">
+        <v>77</v>
+      </c>
+      <c r="B7" s="25" t="n">
         <f aca="false">B5+B6</f>
         <v>9018.075</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="24" t="s">
-        <v>73</v>
-      </c>
-      <c r="B9" s="24"/>
+      <c r="A9" s="26" t="s">
+        <v>78</v>
+      </c>
+      <c r="B9" s="26"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1732,22 +1875,22 @@
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="24" t="s">
-        <v>76</v>
-      </c>
-      <c r="B16" s="24"/>
+      <c r="A16" s="26" t="s">
+        <v>81</v>
+      </c>
+      <c r="B16" s="26"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
-        <v>77</v>
-      </c>
-      <c r="B17" s="27" t="n">
+        <v>82</v>
+      </c>
+      <c r="B17" s="29" t="n">
         <v>1.5</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="B18" s="11" t="n">
         <v>0.1</v>
@@ -1755,102 +1898,203 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="6" t="s">
-        <v>79</v>
-      </c>
-      <c r="B19" s="28" t="n">
+        <v>84</v>
+      </c>
+      <c r="B19" s="30" t="n">
         <v>18</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="3" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="14" t="s">
-        <v>84</v>
-      </c>
-      <c r="B22" s="29" t="n">
+      <c r="A22" s="16" t="s">
+        <v>89</v>
+      </c>
+      <c r="B22" s="31" t="n">
         <f aca="false">$B$17*4</f>
         <v>6</v>
       </c>
-      <c r="C22" s="29" t="n">
+      <c r="C22" s="31" t="n">
         <v>0</v>
       </c>
-      <c r="D22" s="30" t="n">
+      <c r="D22" s="32" t="n">
         <f aca="false">MIN($B$19, C22*(1-$B$18)+B22)</f>
         <v>6</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="14" t="s">
-        <v>85</v>
-      </c>
-      <c r="B23" s="29" t="n">
+      <c r="A23" s="16" t="s">
+        <v>90</v>
+      </c>
+      <c r="B23" s="31" t="n">
         <f aca="false">$B$17*4</f>
         <v>6</v>
       </c>
-      <c r="C23" s="29" t="n">
+      <c r="C23" s="31" t="n">
         <f aca="false">D22</f>
         <v>6</v>
       </c>
-      <c r="D23" s="30" t="n">
+      <c r="D23" s="32" t="n">
         <f aca="false">MIN($B$19, C23*(1-$B$18)+B23)</f>
         <v>11.4</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="14" t="s">
-        <v>86</v>
-      </c>
-      <c r="B24" s="29" t="n">
+      <c r="A24" s="16" t="s">
+        <v>91</v>
+      </c>
+      <c r="B24" s="31" t="n">
         <f aca="false">$B$17*4</f>
         <v>6</v>
       </c>
-      <c r="C24" s="29" t="n">
+      <c r="C24" s="31" t="n">
         <f aca="false">D23</f>
         <v>11.4</v>
       </c>
-      <c r="D24" s="30" t="n">
+      <c r="D24" s="32" t="n">
         <f aca="false">MIN($B$19, C24*(1-$B$18)+B24)</f>
         <v>16.26</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="24" t="s">
-        <v>87</v>
-      </c>
-      <c r="B26" s="24"/>
+      <c r="A26" s="26" t="s">
+        <v>92</v>
+      </c>
+      <c r="B26" s="26"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="B27" s="17" t="n">
+        <v>93</v>
+      </c>
+      <c r="B27" s="19" t="n">
         <f aca="false">(Fuentes!$B$18+Fuentes!$B$19)/Fuentes!$B$17</f>
         <v>0.204606403356745</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="13" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="B28" s="13"/>
       <c r="C28" s="13"/>
       <c r="D28" s="13"/>
       <c r="E28" s="13"/>
     </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="26" t="s">
+        <v>95</v>
+      </c>
+      <c r="B30" s="26"/>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="B31" s="33" t="n">
+        <v>100000</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="B32" s="33" t="n">
+        <v>30000</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="B33" s="34" t="n">
+        <f aca="false">B31+B32*12</f>
+        <v>460000</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="B34" s="34" t="n">
+        <f aca="false">B32*12</f>
+        <v>360000</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="B36" s="11" t="n">
+        <v>0.08</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="B37" s="35" t="n">
+        <f aca="false">B33/B36</f>
+        <v>5750000</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="B38" s="35" t="n">
+        <f aca="false">B34/B36</f>
+        <v>4500000</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="13" t="s">
+        <v>103</v>
+      </c>
+      <c r="B39" s="13"/>
+      <c r="C39" s="13"/>
+      <c r="D39" s="13"/>
+      <c r="E39" s="13"/>
+    </row>
+    <row r="41" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="B41" s="11" t="n">
+        <v>0.35</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="24" t="s">
+        <v>105</v>
+      </c>
+      <c r="B42" s="25" t="n">
+        <f aca="false">B7*B41</f>
+        <v>3156.32625</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="54.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A43" s="36" t="s">
+        <v>106</v>
+      </c>
+      <c r="B43" s="36"/>
+      <c r="C43" s="36"/>
+      <c r="D43" s="36"/>
+      <c r="E43" s="36"/>
+    </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="10">
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A2:E2"/>
     <mergeCell ref="A4:B4"/>
@@ -1858,6 +2102,9 @@
     <mergeCell ref="A16:B16"/>
     <mergeCell ref="A26:B26"/>
     <mergeCell ref="A28:E28"/>
+    <mergeCell ref="A30:B30"/>
+    <mergeCell ref="A39:E39"/>
+    <mergeCell ref="A43:E43"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -1883,7 +2130,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>90</v>
+        <v>107</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1891,7 +2138,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>91</v>
+        <v>108</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -1902,23 +2149,23 @@
         <v>2</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>92</v>
+        <v>109</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>93</v>
+        <v>110</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>94</v>
+        <v>111</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>95</v>
+        <v>112</v>
       </c>
       <c r="B5" s="8" t="n">
         <v>0.15</v>
       </c>
-      <c r="C5" s="17" t="n">
+      <c r="C5" s="19" t="n">
         <f aca="false">Fuentes!$B$27</f>
         <v>0.25</v>
       </c>
@@ -1928,12 +2175,12 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>96</v>
+        <v>113</v>
       </c>
       <c r="B6" s="8" t="n">
         <v>0.75</v>
       </c>
-      <c r="C6" s="17" t="n">
+      <c r="C6" s="19" t="n">
         <f aca="false">Fuentes!$B$28</f>
         <v>0.85</v>
       </c>
@@ -1943,12 +2190,12 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="B7" s="8" t="n">
         <v>0.1</v>
       </c>
-      <c r="C7" s="17" t="n">
+      <c r="C7" s="19" t="n">
         <f aca="false">Fuentes!$B$29</f>
         <v>0.2</v>
       </c>
@@ -1957,52 +2204,52 @@
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="14" t="s">
-        <v>97</v>
-      </c>
-      <c r="B9" s="31" t="n">
+      <c r="A9" s="16" t="s">
+        <v>114</v>
+      </c>
+      <c r="B9" s="37" t="n">
         <f aca="false">Fuentes!$B$17*B5*B6*B7</f>
         <v>1233.3375</v>
       </c>
-      <c r="C9" s="31" t="n">
+      <c r="C9" s="37" t="n">
         <f aca="false">Fuentes!$B$17*C5*C6*C7</f>
         <v>4659.275</v>
       </c>
-      <c r="D9" s="31" t="n">
+      <c r="D9" s="37" t="n">
         <f aca="false">Fuentes!$B$17*D5*D6*D7</f>
         <v>10360.035</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="14" t="s">
-        <v>98</v>
-      </c>
-      <c r="B10" s="31" t="n">
+      <c r="A10" s="16" t="s">
+        <v>115</v>
+      </c>
+      <c r="B10" s="37" t="n">
         <f aca="false">Fuentes!$B$14*Fuentes!$B$16*B6*B7</f>
         <v>1923</v>
       </c>
-      <c r="C10" s="31" t="n">
+      <c r="C10" s="37" t="n">
         <f aca="false">Fuentes!$B$14*Fuentes!$B$16*C6*C7</f>
         <v>4358.8</v>
       </c>
-      <c r="D10" s="31" t="n">
+      <c r="D10" s="37" t="n">
         <f aca="false">Fuentes!$B$14*Fuentes!$B$16*D6*D7</f>
         <v>6922.80000000001</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="22" t="s">
-        <v>99</v>
-      </c>
-      <c r="B11" s="23" t="n">
+      <c r="A11" s="24" t="s">
+        <v>116</v>
+      </c>
+      <c r="B11" s="25" t="n">
         <f aca="false">B9+B10</f>
         <v>3156.3375</v>
       </c>
-      <c r="C11" s="23" t="n">
+      <c r="C11" s="25" t="n">
         <f aca="false">C9+C10</f>
         <v>9018.075</v>
       </c>
-      <c r="D11" s="23" t="n">
+      <c r="D11" s="25" t="n">
         <f aca="false">D9+D10</f>
         <v>17282.835</v>
       </c>

</xml_diff>

<commit_message>
Add revenue projection and illustrative valuation range sheet
New 'Valoracion' sheet: projects revenue from the existing solo-operator
capacity table at the proposed $100k setup / $30k/mo pricing, then
applies boutique-services valuation multiples (0.5x-1.5x ARR, explicitly
not SaaS multiples since the automation is bespoke, not owned IP) to give
an illustrative business value range. Heavily caveated as directional,
not a formal valuation.
</commit_message>
<xml_diff>
--- a/modelo-mercado-pymes-mexico.xlsx
+++ b/modelo-mercado-pymes-mexico.xlsx
@@ -13,6 +13,7 @@
     <sheet name="Via B" sheetId="3" state="visible" r:id="rId5"/>
     <sheet name="Resumen" sheetId="4" state="visible" r:id="rId6"/>
     <sheet name="Sensibilidad" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="Valoracion" sheetId="6" state="visible" r:id="rId8"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -24,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="133">
   <si>
     <t xml:space="preserve">Fuentes y supuestos — modelo de mercado de PYMEs en México</t>
   </si>
@@ -375,18 +376,73 @@
   </si>
   <si>
     <t xml:space="preserve">SOM TOTAL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Valoración — proyección de ingresos y rango de valor del negocio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ilustrativo, NO es una valoración formal: no incorpora margen real, estructura de costos ni contratos. Útil para ver el orden de magnitud, no para negociar una venta. El techo aquí es tu capacidad operativa (hoja 'Resumen'), no el tamaño de mercado — el mercado ya es muchas veces mayor que lo que puedes atender solo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Proyección de ingresos (usa la capacidad operativa ya modelada en 'Resumen')</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nuevos clientes
+instalados</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cartera al
+inicio del año</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cartera al
+cierre del año</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ingreso por
+setup (MXN)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ingreso recurrente
+promedio del año (MXN)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ingreso total
+del año (MXN)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ingreso recurrente anualizado de salida (ARR) al cierre del Año 3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Múltiplos de valoración (supuestos)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Negocio de servicios boutique, un solo operador, alto riesgo de dependencia de una persona clave (si tú no estás, ¿el negocio sigue?). No es una empresa de software (TINO no es tuyo, la automatización es a la medida) — no apliques múltiplos de SaaS (5–10x ARR). Rangos típicos para consultoría boutique de una persona: 0.5x–1.5x del ingreso recurrente anualizado.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Escenario</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Múltiplo sobre ARR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Valor estimado (MXN)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nota: hoy tienes un cliente real operando — no una cartera de varios clientes con historial. Este rango es hacia dónde apunta el negocio si la proyección de capacidad se cumple, no lo que vale hoy. Lo que más sube el múltiplo real, si algún día quieres vender o atraer socios: que el sistema funcione sin que tú estés en cada cuenta (documentación, un segundo operador, procesos repetibles), y contratos de monitoreo firmados a 12+ meses en vez de mes a mes.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="5">
+  <numFmts count="6">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="#,##0"/>
     <numFmt numFmtId="166" formatCode="0.0%"/>
     <numFmt numFmtId="167" formatCode="#,##0.0"/>
     <numFmt numFmtId="168" formatCode="\$#,##0"/>
+    <numFmt numFmtId="169" formatCode="0.00\x"/>
   </numFmts>
   <fonts count="19">
     <font>
@@ -605,7 +661,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="41">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -755,6 +811,18 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="14" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="11" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2267,4 +2335,268 @@
     <oddFooter/>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:G19"/>
+  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="2" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="20"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="26" t="s">
+        <v>119</v>
+      </c>
+      <c r="B4" s="26"/>
+      <c r="C4" s="26"/>
+      <c r="D4" s="26"/>
+      <c r="E4" s="26"/>
+      <c r="F4" s="26"/>
+      <c r="G4" s="26"/>
+    </row>
+    <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="16" t="str">
+        <f aca="false">Resumen!A22</f>
+        <v>Año 1</v>
+      </c>
+      <c r="B6" s="38" t="n">
+        <f aca="false">Resumen!B22</f>
+        <v>6</v>
+      </c>
+      <c r="C6" s="38" t="n">
+        <f aca="false">Resumen!C22</f>
+        <v>0</v>
+      </c>
+      <c r="D6" s="38" t="n">
+        <f aca="false">Resumen!D22</f>
+        <v>6</v>
+      </c>
+      <c r="E6" s="35" t="n">
+        <f aca="false">B6*Resumen!$B$31</f>
+        <v>600000</v>
+      </c>
+      <c r="F6" s="35" t="n">
+        <f aca="false">AVERAGE(C6,D6)*Resumen!$B$32*12</f>
+        <v>1080000</v>
+      </c>
+      <c r="G6" s="39" t="n">
+        <f aca="false">E6+F6</f>
+        <v>1680000</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="16" t="str">
+        <f aca="false">Resumen!A23</f>
+        <v>Año 2</v>
+      </c>
+      <c r="B7" s="38" t="n">
+        <f aca="false">Resumen!B23</f>
+        <v>6</v>
+      </c>
+      <c r="C7" s="38" t="n">
+        <f aca="false">Resumen!C23</f>
+        <v>6</v>
+      </c>
+      <c r="D7" s="38" t="n">
+        <f aca="false">Resumen!D23</f>
+        <v>11.4</v>
+      </c>
+      <c r="E7" s="35" t="n">
+        <f aca="false">B7*Resumen!$B$31</f>
+        <v>600000</v>
+      </c>
+      <c r="F7" s="35" t="n">
+        <f aca="false">AVERAGE(C7,D7)*Resumen!$B$32*12</f>
+        <v>3132000</v>
+      </c>
+      <c r="G7" s="39" t="n">
+        <f aca="false">E7+F7</f>
+        <v>3732000</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="16" t="str">
+        <f aca="false">Resumen!A24</f>
+        <v>Año 3</v>
+      </c>
+      <c r="B8" s="38" t="n">
+        <f aca="false">Resumen!B24</f>
+        <v>6</v>
+      </c>
+      <c r="C8" s="38" t="n">
+        <f aca="false">Resumen!C24</f>
+        <v>11.4</v>
+      </c>
+      <c r="D8" s="38" t="n">
+        <f aca="false">Resumen!D24</f>
+        <v>16.26</v>
+      </c>
+      <c r="E8" s="35" t="n">
+        <f aca="false">B8*Resumen!$B$31</f>
+        <v>600000</v>
+      </c>
+      <c r="F8" s="35" t="n">
+        <f aca="false">AVERAGE(C8,D8)*Resumen!$B$32*12</f>
+        <v>4978800</v>
+      </c>
+      <c r="G8" s="39" t="n">
+        <f aca="false">E8+F8</f>
+        <v>5578800</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="6" t="s">
+        <v>126</v>
+      </c>
+      <c r="B10" s="34" t="n">
+        <f aca="false">Resumen!D24*Resumen!$B$32*12</f>
+        <v>5853600</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="26" t="s">
+        <v>127</v>
+      </c>
+      <c r="B12" s="26"/>
+      <c r="C12" s="26"/>
+    </row>
+    <row r="13" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="13" t="s">
+        <v>128</v>
+      </c>
+      <c r="B13" s="13"/>
+      <c r="C13" s="13"/>
+      <c r="D13" s="13"/>
+      <c r="E13" s="13"/>
+      <c r="F13" s="13"/>
+      <c r="G13" s="13"/>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="16" t="s">
+        <v>109</v>
+      </c>
+      <c r="B15" s="40" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C15" s="34" t="n">
+        <f aca="false">$B$10*B15</f>
+        <v>2926800</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="16" t="s">
+        <v>110</v>
+      </c>
+      <c r="B16" s="40" t="n">
+        <v>1</v>
+      </c>
+      <c r="C16" s="34" t="n">
+        <f aca="false">$B$10*B16</f>
+        <v>5853600</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="16" t="s">
+        <v>111</v>
+      </c>
+      <c r="B17" s="40" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="C17" s="34" t="n">
+        <f aca="false">$B$10*B17</f>
+        <v>8780400</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="54.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="36" t="s">
+        <v>132</v>
+      </c>
+      <c r="B19" s="36"/>
+      <c r="C19" s="36"/>
+      <c r="D19" s="36"/>
+      <c r="E19" s="36"/>
+      <c r="F19" s="36"/>
+      <c r="G19" s="36"/>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A4:G4"/>
+    <mergeCell ref="A12:C12"/>
+    <mergeCell ref="A13:G13"/>
+    <mergeCell ref="A19:G19"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add scale-to-$30M feasibility sheet
New 'Escala30M' sheet: reverse-engineers the monitoring cartera and
team size needed to sustain $30M MXN/year, then projects a year-by-year
trajectory under a ~1-operator-per-year hiring ramp. Revenue-only model
(no cost/margin) - explicitly flagged as answering "is the revenue
reachable," not "is it a good business at that scale."
</commit_message>
<xml_diff>
--- a/modelo-mercado-pymes-mexico.xlsx
+++ b/modelo-mercado-pymes-mexico.xlsx
@@ -14,6 +14,7 @@
     <sheet name="Resumen" sheetId="4" state="visible" r:id="rId6"/>
     <sheet name="Sensibilidad" sheetId="5" state="visible" r:id="rId7"/>
     <sheet name="Valoracion" sheetId="6" state="visible" r:id="rId8"/>
+    <sheet name="Escala30M" sheetId="7" state="visible" r:id="rId9"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="133">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="212" uniqueCount="151">
   <si>
     <t xml:space="preserve">Fuentes y supuestos — modelo de mercado de PYMEs en México</t>
   </si>
@@ -430,6 +431,66 @@
   </si>
   <si>
     <t xml:space="preserve">Nota: hoy tienes un cliente real operando — no una cartera de varios clientes con historial. Este rango es hacia dónde apunta el negocio si la proyección de capacidad se cumple, no lo que vale hoy. Lo que más sube el múltiplo real, si algún día quieres vender o atraer socios: que el sistema funcione sin que tú estés en cada cuenta (documentación, un segundo operador, procesos repetibles), y contratos de monitoreo firmados a 12+ meses en vez de mes a mes.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">¿Es factible escalar a $30M MXN/año?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Este modelo sólo proyecta ingreso, no utilidad: no incluye sueldos de los operadores nuevos, costo de adquisición de clientes, ni gastos de operación. Responde '¿el ingreso es alcanzable?', no '¿es un buen negocio a esa escala?'.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Objetivo de ingreso anual (MXN)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cartera en monitoreo necesaria (asumiendo que el ingreso viene sobre todo de mensualidades)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Operadores equivalentes necesarios (usando tu propio techo por operador de 'Resumen')</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Clientes nuevos por año que hacen falta sólo para reponer bajas en estado estable (cartera × tasa de cancelación)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Trayectoria — ¿cuánto tarda en llegar, contratando ~1 operador nuevo por año?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">'Operadores activos' es un supuesto editable por año (empieza en ti solo). Cada operador aporta la misma capacidad que la tuya en 'Resumen': 1.5 clientes nuevos instalados por trimestre, techo de 18 en cartera. Es una simplificación — en la práctica un operador nuevo tarda en llegar a ese ritmo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Operadores
+activos (supuesto)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Techo de
+cartera</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cartera al
+inicio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cartera al
+cierre</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ingreso recurrente
+del año (MXN)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ingreso por
+setups (MXN)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Año 4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Año 5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Año 6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nota: la meta de mercado no es el cuello de botella — necesitas ~80-100 clientes activos de un mercado obtenible de ~9,000 (hoja 'Resumen'). El cuello de botella real es operativo: pasar de consultor solo a un equipo de 5-6 personas sin perder la calidad que hace verificable el trabajo (auditoría v1/v2), y el ritmo de ventas necesario para llenar esa capacidad nueva cada año. Este modelo no dice si la economía por operador (sueldo vs. ingreso que genera) funciona — sólo que el ingreso agregado es alcanzable.</t>
   </si>
 </sst>
 </file>
@@ -661,7 +722,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="43">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -823,6 +884,14 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="169" fontId="11" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2599,4 +2668,382 @@
     <oddFooter/>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:I19"/>
+  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="4" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="20"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+      <c r="I1" s="1"/>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+      <c r="H2" s="2"/>
+      <c r="I2" s="2"/>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="16" t="s">
+        <v>135</v>
+      </c>
+      <c r="B4" s="33" t="n">
+        <v>30000000</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="B5" s="41" t="n">
+        <f aca="false">B4/(Resumen!$B$32*12)</f>
+        <v>83.3333333333333</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="B6" s="42" t="n">
+        <f aca="false">ROUNDUP(B5/Resumen!$B$19,0)</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="4" t="s">
+        <v>138</v>
+      </c>
+      <c r="B7" s="41" t="n">
+        <f aca="false">B5*Resumen!$B$18</f>
+        <v>8.33333333333333</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="26" t="s">
+        <v>139</v>
+      </c>
+      <c r="B9" s="26"/>
+      <c r="C9" s="26"/>
+      <c r="D9" s="26"/>
+      <c r="E9" s="26"/>
+      <c r="F9" s="26"/>
+      <c r="G9" s="26"/>
+      <c r="H9" s="26"/>
+      <c r="I9" s="26"/>
+    </row>
+    <row r="10" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="13" t="s">
+        <v>140</v>
+      </c>
+      <c r="B10" s="13"/>
+      <c r="C10" s="13"/>
+      <c r="D10" s="13"/>
+      <c r="E10" s="13"/>
+      <c r="F10" s="13"/>
+      <c r="G10" s="13"/>
+      <c r="H10" s="13"/>
+      <c r="I10" s="13"/>
+    </row>
+    <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>144</v>
+      </c>
+      <c r="G11" s="3" t="s">
+        <v>145</v>
+      </c>
+      <c r="H11" s="3" t="s">
+        <v>146</v>
+      </c>
+      <c r="I11" s="3" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="16" t="s">
+        <v>89</v>
+      </c>
+      <c r="B12" s="30" t="n">
+        <v>1</v>
+      </c>
+      <c r="C12" s="31" t="n">
+        <f aca="false">B12*Resumen!$B$17*4</f>
+        <v>6</v>
+      </c>
+      <c r="D12" s="31" t="n">
+        <f aca="false">B12*Resumen!$B$19</f>
+        <v>18</v>
+      </c>
+      <c r="E12" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" s="32" t="n">
+        <f aca="false">MIN(D12, E12*(1-Resumen!$B$18)+C12)</f>
+        <v>6</v>
+      </c>
+      <c r="G12" s="35" t="n">
+        <f aca="false">AVERAGE(E12,F12)*Resumen!$B$32*12</f>
+        <v>1080000</v>
+      </c>
+      <c r="H12" s="35" t="n">
+        <f aca="false">C12*Resumen!$B$31</f>
+        <v>600000</v>
+      </c>
+      <c r="I12" s="39" t="n">
+        <f aca="false">G12+H12</f>
+        <v>1680000</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="16" t="s">
+        <v>90</v>
+      </c>
+      <c r="B13" s="30" t="n">
+        <v>2</v>
+      </c>
+      <c r="C13" s="31" t="n">
+        <f aca="false">B13*Resumen!$B$17*4</f>
+        <v>12</v>
+      </c>
+      <c r="D13" s="31" t="n">
+        <f aca="false">B13*Resumen!$B$19</f>
+        <v>36</v>
+      </c>
+      <c r="E13" s="31" t="n">
+        <f aca="false">F12</f>
+        <v>6</v>
+      </c>
+      <c r="F13" s="32" t="n">
+        <f aca="false">MIN(D13, E13*(1-Resumen!$B$18)+C13)</f>
+        <v>17.4</v>
+      </c>
+      <c r="G13" s="35" t="n">
+        <f aca="false">AVERAGE(E13,F13)*Resumen!$B$32*12</f>
+        <v>4212000</v>
+      </c>
+      <c r="H13" s="35" t="n">
+        <f aca="false">C13*Resumen!$B$31</f>
+        <v>1200000</v>
+      </c>
+      <c r="I13" s="39" t="n">
+        <f aca="false">G13+H13</f>
+        <v>5412000</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="16" t="s">
+        <v>91</v>
+      </c>
+      <c r="B14" s="30" t="n">
+        <v>3</v>
+      </c>
+      <c r="C14" s="31" t="n">
+        <f aca="false">B14*Resumen!$B$17*4</f>
+        <v>18</v>
+      </c>
+      <c r="D14" s="31" t="n">
+        <f aca="false">B14*Resumen!$B$19</f>
+        <v>54</v>
+      </c>
+      <c r="E14" s="31" t="n">
+        <f aca="false">F13</f>
+        <v>17.4</v>
+      </c>
+      <c r="F14" s="32" t="n">
+        <f aca="false">MIN(D14, E14*(1-Resumen!$B$18)+C14)</f>
+        <v>33.66</v>
+      </c>
+      <c r="G14" s="35" t="n">
+        <f aca="false">AVERAGE(E14,F14)*Resumen!$B$32*12</f>
+        <v>9190800</v>
+      </c>
+      <c r="H14" s="35" t="n">
+        <f aca="false">C14*Resumen!$B$31</f>
+        <v>1800000</v>
+      </c>
+      <c r="I14" s="39" t="n">
+        <f aca="false">G14+H14</f>
+        <v>10990800</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="16" t="s">
+        <v>147</v>
+      </c>
+      <c r="B15" s="30" t="n">
+        <v>4</v>
+      </c>
+      <c r="C15" s="31" t="n">
+        <f aca="false">B15*Resumen!$B$17*4</f>
+        <v>24</v>
+      </c>
+      <c r="D15" s="31" t="n">
+        <f aca="false">B15*Resumen!$B$19</f>
+        <v>72</v>
+      </c>
+      <c r="E15" s="31" t="n">
+        <f aca="false">F14</f>
+        <v>33.66</v>
+      </c>
+      <c r="F15" s="32" t="n">
+        <f aca="false">MIN(D15, E15*(1-Resumen!$B$18)+C15)</f>
+        <v>54.294</v>
+      </c>
+      <c r="G15" s="35" t="n">
+        <f aca="false">AVERAGE(E15,F15)*Resumen!$B$32*12</f>
+        <v>15831720</v>
+      </c>
+      <c r="H15" s="35" t="n">
+        <f aca="false">C15*Resumen!$B$31</f>
+        <v>2400000</v>
+      </c>
+      <c r="I15" s="39" t="n">
+        <f aca="false">G15+H15</f>
+        <v>18231720</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="16" t="s">
+        <v>148</v>
+      </c>
+      <c r="B16" s="30" t="n">
+        <v>5</v>
+      </c>
+      <c r="C16" s="31" t="n">
+        <f aca="false">B16*Resumen!$B$17*4</f>
+        <v>30</v>
+      </c>
+      <c r="D16" s="31" t="n">
+        <f aca="false">B16*Resumen!$B$19</f>
+        <v>90</v>
+      </c>
+      <c r="E16" s="31" t="n">
+        <f aca="false">F15</f>
+        <v>54.294</v>
+      </c>
+      <c r="F16" s="32" t="n">
+        <f aca="false">MIN(D16, E16*(1-Resumen!$B$18)+C16)</f>
+        <v>78.8646</v>
+      </c>
+      <c r="G16" s="35" t="n">
+        <f aca="false">AVERAGE(E16,F16)*Resumen!$B$32*12</f>
+        <v>23968548</v>
+      </c>
+      <c r="H16" s="35" t="n">
+        <f aca="false">C16*Resumen!$B$31</f>
+        <v>3000000</v>
+      </c>
+      <c r="I16" s="39" t="n">
+        <f aca="false">G16+H16</f>
+        <v>26968548</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="16" t="s">
+        <v>149</v>
+      </c>
+      <c r="B17" s="30" t="n">
+        <v>6</v>
+      </c>
+      <c r="C17" s="31" t="n">
+        <f aca="false">B17*Resumen!$B$17*4</f>
+        <v>36</v>
+      </c>
+      <c r="D17" s="31" t="n">
+        <f aca="false">B17*Resumen!$B$19</f>
+        <v>108</v>
+      </c>
+      <c r="E17" s="31" t="n">
+        <f aca="false">F16</f>
+        <v>78.8646</v>
+      </c>
+      <c r="F17" s="32" t="n">
+        <f aca="false">MIN(D17, E17*(1-Resumen!$B$18)+C17)</f>
+        <v>106.97814</v>
+      </c>
+      <c r="G17" s="35" t="n">
+        <f aca="false">AVERAGE(E17,F17)*Resumen!$B$32*12</f>
+        <v>33451693.2</v>
+      </c>
+      <c r="H17" s="35" t="n">
+        <f aca="false">C17*Resumen!$B$31</f>
+        <v>3600000</v>
+      </c>
+      <c r="I17" s="39" t="n">
+        <f aca="false">G17+H17</f>
+        <v>37051693.2</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="54.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="36" t="s">
+        <v>150</v>
+      </c>
+      <c r="B19" s="36"/>
+      <c r="C19" s="36"/>
+      <c r="D19" s="36"/>
+      <c r="E19" s="36"/>
+      <c r="F19" s="36"/>
+      <c r="G19" s="36"/>
+      <c r="H19" s="36"/>
+      <c r="I19" s="36"/>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A2:I2"/>
+    <mergeCell ref="A9:I9"/>
+    <mergeCell ref="A10:I10"/>
+    <mergeCell ref="A19:I19"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>